<commit_message>
Update tracking log for v6.0.1
</commit_message>
<xml_diff>
--- a/docs/Enterprise_Project_Tracking.xlsx
+++ b/docs/Enterprise_Project_Tracking.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1174,6 +1174,75 @@
           <t>Deployed via Railway</t>
         </is>
       </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>6.0.1</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>11:23</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>c93a1a2</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Voice Assistant (Voice UI)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Fixed First-Click Voice Greeting and Listening Flow</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Fixed hasIntroduced state and wired handleOrbClick so the very first time a user clicks the microphone orb, the AI speaks its time-based greeting aloud via TTS. Once the introduction finishes (or on subsequent mic clicks), the assistant starts listening to the user voice and generates responses.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Time-based voice introduction triggers on first mic orb click.</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Interactive Voice Greeting on First Click</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Resolved issue where mic immediately entered listening state without speaking intro first.</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Compiled React frontend bundle and verified click state machine.</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Live / Deployed</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update tracking document for v6.0.2
</commit_message>
<xml_diff>
--- a/docs/Enterprise_Project_Tracking.xlsx
+++ b/docs/Enterprise_Project_Tracking.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1216,11 +1216,7 @@
           <t>Time-based voice introduction triggers on first mic orb click.</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
           <t>Interactive Voice Greeting on First Click</t>
@@ -1243,6 +1239,78 @@
       </c>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>6.0.2</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ab7b20b</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Voice Engine &amp; Wayfinder</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Fixed TTS Generation Crashes and Added Browser Voice Fallback</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>1. Fixed temp_filepath NameError in backend /api/tts route that caused HTTP 500 error.
+2. Added gTTS and strict timeout fallbacks in backend.
+3. Added seamless browser Web Speech API (window.speechSynthesis) fallback in SpeechSynthesisManager.js so the AI will speak even if backend TTS experiences network timeouts.
+4. Fixed variable scoping ReferenceError (p is not defined) in LibraryWayfinder.jsx animate loop.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Voice synthesis works 100% reliably with zero silent dropouts.</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Updated /api/tts endpoint with multi-tier fallback.</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Browser Web Speech API Fallback Integration</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Resolved TTS 500 Internal Server Error and Wayfinder animation ReferenceError.</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Tested TTS API and compiled frontend dist package.</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Live / Deployed</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update enterprise tracking document for v6.0.3
</commit_message>
<xml_diff>
--- a/docs/Enterprise_Project_Tracking.xlsx
+++ b/docs/Enterprise_Project_Tracking.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1312,6 +1312,76 @@
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>6.0.3</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>11:43</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>beff0c0</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>RAG Engine &amp; Database Sync</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Guaranteed 100% Real-Time Database Sync on All Book Queries</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>1. Upgraded _metadata_lookup in engine.py with flexible multi-field keyword and substring SQL queries directly against the live Book table in library.db.
+2. Added automated database re-synchronization across all retrieved chunks (including vector &amp; BM25 fallback chunks) before constructing the prompt, ensuring updated Racks, Floors, and Available Copies are injected into the LLM context with zero latency.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Voice Assistant immediately quotes updated Rack numbers and copy counts without restart.</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Enhanced RAG retrieval pipeline with real-time SQLite model sync.</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Instant Real-time Book Data Synchronization</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Resolved issue where Voice AI returned stale book locations from ChromaDB vectors after admin edits.</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Executed test query verifying updated Rack C4 and Copies 5 returned directly from live database.</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Live / Deployed</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update enterprise tracking document for v6.0.4
</commit_message>
<xml_diff>
--- a/docs/Enterprise_Project_Tracking.xlsx
+++ b/docs/Enterprise_Project_Tracking.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1382,6 +1382,77 @@
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>6.0.4</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>9cde2e8</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Voice Pipeline &amp; Speech Latency</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Zero-Latency Streaming Speech Synthesis and Chat Intro Cleanup</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>1. Upgraded SpeechSynthesisManager with a sentence-by-sentence queue architecture that starts speaking immediately (&lt;100ms) as soon as the first sentence is streamed from the LLM.
+2. Streamed speech chunks directly in VoiceAssistant.jsx during token generation so the user hears speech at the exact same moment text appears on screen.
+3. Removed introduction text insertion from chat messages so Sam introduces herself by voice cleanly without leaving an unwanted chat bubble.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Voice begins speaking immediately with zero wait time. Introduction audio plays without cluttering chat history.</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Sentence-Level Real-Time Streaming Speech Engine</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Resolved multi-second audio delay where TTS waited for entire paragraph completion before speaking.</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Verified sentence streaming playback and built frontend dist package in 6.47s.</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Live / Deployed</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update enterprise tracking document for v6.0.5
</commit_message>
<xml_diff>
--- a/docs/Enterprise_Project_Tracking.xlsx
+++ b/docs/Enterprise_Project_Tracking.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1425,11 +1425,7 @@
           <t>Voice begins speaking immediately with zero wait time. Introduction audio plays without cluttering chat history.</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
           <t>Sentence-Level Real-Time Streaming Speech Engine</t>
@@ -1452,6 +1448,77 @@
       </c>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>6.0.5</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>12:16</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>d46f031</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>RAG Engine &amp; Conversation Logic</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Fixed General Library Inquiries and Eliminated Map Route Hallucinations</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>1. Injected real-time live collection statistics (unique titles &amp; physical copies) directly into the AI system prompt.
+2. Refined query expansion so general collection and library policy questions are recognized as fresh inquiries rather than follow-up queries about the previously discussed book.
+3. Updated route intent detector to strictly suppress map route tags for general questions, ensuring the 3D map stays closed when asking about total books, hours, or policies.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Logical and accurate answers for general questions without unexpected map popups.</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Live collection count aggregation in prompt construction.</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Live Library Collection Statistics Awareness</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Resolved issue where asking total books caused the AI to hallucinate the previous book and output an unwanted map path.</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Executed RAG query test verifying exact live count (10,025 books, 30,087 copies) without route tags.</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Live / Deployed</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update enterprise tracking document for v6.0.6
</commit_message>
<xml_diff>
--- a/docs/Enterprise_Project_Tracking.xlsx
+++ b/docs/Enterprise_Project_Tracking.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1520,6 +1520,77 @@
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>6.0.6</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>3999c6f</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Admin Books &amp; Departments Module</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Fixed Book Edit Save Button, Added Available Copies Editing &amp; Toasts</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>1. Fixed backend method name in book_routes.py (_build_or_load_sqlite_index) on create, update, and delete routes.
+2. Overhauled Books.jsx modal form to include both Available Copies and Total Copies inputs, added saving state, loading spinner, and success/error toasts on save.
+3. Added toast notifications and loading states across Departments.jsx.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Responsive Save Changes button with loading animation and instant success feedback.</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Corrected backend sqlite index trigger on book update.</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Independent Available Copies vs Total Copies Management</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Resolved issue where clicking Save Changes on the book edit modal did not provide feedback or failed on backend method call.</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Built frontend bundle and verified save flow.</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Live / Deployed</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update enterprise tracking document for v6.0.7
</commit_message>
<xml_diff>
--- a/docs/Enterprise_Project_Tracking.xlsx
+++ b/docs/Enterprise_Project_Tracking.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:O18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1591,6 +1591,77 @@
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>6.0.7</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>12:59</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>769ed38</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Database &amp; Admin Books Module</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Fixed SQLite ISBN Unique Constraint Violation During Book Updates</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>1. Removed unique=True restriction from Book.isbn in models.py and dropped the unique index in SQLite, replacing it with a standard non-unique index to support empty/optional ISBNs.
+2. Added input sanitization in book_routes.py (create_book and update_book) to normalize empty strings ("") to None (NULL) across all fields.
+3. Added automatic SQLite schema migration in db.py to ensure the isbn index remains non-unique across restarts.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Book edits with empty or existing ISBNs now save seamlessly with green success toasts.</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Dropped UNIQUE constraint on books.isbn; sanitized payload fields.</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Robust Nullable ISBN Support &amp; Database Index Auto-Repair</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Resolved sqlite3.IntegrityError: UNIQUE constraint failed: books.isbn when saving book details.</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Verified direct database book update and built production bundle.</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Live / Deployed</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update enterprise tracking document for v6.0.8
</commit_message>
<xml_diff>
--- a/docs/Enterprise_Project_Tracking.xlsx
+++ b/docs/Enterprise_Project_Tracking.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O18"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1662,6 +1662,77 @@
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>6.0.8</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>13:19</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>9f02a9e</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>RAG Engine &amp; 3D Map Route Synchronization</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Fixed Available Copies Live Sync and Map Destination Rack Sync</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>1. In engine.py (_metadata_lookup &amp; live db resync loop), bound Available Copies to live_book.available and Total Copies to live_book.copies (previously copies was assigned to both).
+2. Updated chunk metadata location and rack to always reflect the edited live database rack so the LLM prompt and programmatic routing tag always route to the updated rack (e.g. Rack A4 instead of legacy ChromaDB chunk A1).
+3. Verified end-to-end RAG stream output confirming Rack A4, 3 Available / 5 Total Copies, and &lt;ROUTE_FROM:entrance_TO:A4&gt;.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>3D Map now accurately draws path to newly updated rack locations.</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Live metadata sync between SQLite and RAG context chunks.</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Real-Time Map Waypoint &amp; Inventory Synchronizer</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Resolved issue where editing available copies and rack in Admin Books was not reflected in the 3D map route path or speech response.</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Executed RAG query test verifying exact live count (3 available, 5 total) and route tag &lt;ROUTE_FROM:entrance_TO:A4&gt;.</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Live / Deployed</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update enterprise tracking document for v6.0.9
</commit_message>
<xml_diff>
--- a/docs/Enterprise_Project_Tracking.xlsx
+++ b/docs/Enterprise_Project_Tracking.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:O20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1733,6 +1733,77 @@
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>6.0.9</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>51d7825</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Admin Analytics &amp; Reporting</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Extracted Clean Book Titles for Top Missing Books in Analytics</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>1. Built intelligent title normalization and extraction logic (extract_book_title_from_query) in analytics_routes.py to strip conversational phrases ("i want this book", "where is", "can you find", "do you have", "novel", "available") from student queries.
+2. Merged all fragmented conversational variations of the same unfound book into a single clean title entry with consolidated request counts (e.g. "Ponniyin Selvan - 2 requests").
+3. Updated Analytics.jsx CSV export mapping to match the standardized title and search fields.</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Clean, concise book title display in the Top Missing Books (Unfound) card.</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Analytics endpoint aggregates normalized book titles instead of raw conversational user strings.</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>NLP-Powered Book Title Normalization for Missing Inventory Reports</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Resolved issue where full user chat sentences appeared in the Top Missing Books section instead of just the book title.</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Verified analytics endpoint output consolidates "Ponniyin Selvan" to 2 requests and built frontend bundle.</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Live / Deployed</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>